<commit_message>
update with optimized pricing swing and adaptive sweep to ensure the opmitized price is based on the requirement needs of the statistic basis
</commit_message>
<xml_diff>
--- a/routes.xlsx
+++ b/routes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nash/Desktop/Flight_Fare_Prediction_Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B844EB78-E8CC-9043-9D90-DC3C69C4D4FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6209906E-2E45-4D40-8D3D-9483EFF19CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3740" yWindow="3200" windowWidth="28040" windowHeight="17180" xr2:uid="{8E0163F9-584F-5D4F-AF3A-A91933E133B5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="13">
   <si>
     <t>route_id</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t>NRT</t>
+  </si>
+  <si>
+    <t>BTU</t>
   </si>
 </sst>
 </file>
@@ -449,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F133F9E3-23E8-EB44-A2DD-59737A7E2297}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -564,6 +567,20 @@
         <v>400</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>108</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9">
+        <v>180</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>